<commit_message>
Upload AI auditlog week 3
</commit_message>
<xml_diff>
--- a/SWR302_SE20A07_DE190512_MaiVanLuong.xlsx
+++ b/SWR302_SE20A07_DE190512_MaiVanLuong.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SU26\SWR\auditlog\ai-audit-log-MaiLuong1906\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DEC51BD-56AD-4787-92C6-ECCABC4BF8F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8439F8C0-8CD0-4FC0-B728-4D74B2D98661}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Metadata &amp; Summary" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="126">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="187">
   <si>
     <t>AI AUDIT LOG - METADATA &amp; SUMMARY</t>
   </si>
@@ -758,6 +758,208 @@
   </si>
   <si>
     <t>Gemini</t>
+  </si>
+  <si>
+    <t>Tư vấn thiết kế Use Case, phân tích scope</t>
+  </si>
+  <si>
+    <t>10 lần (tuần 1-2)</t>
+  </si>
+  <si>
+    <t>Phân tích UML relationships, tư vấn scope</t>
+  </si>
+  <si>
+    <t>Claude (claude.ai)</t>
+  </si>
+  <si>
+    <t>Thiết kế Context Diagram, DFD-0/1/2, tư vấn data flow</t>
+  </si>
+  <si>
+    <t>16 lần (tuần 3)</t>
+  </si>
+  <si>
+    <t>Giải thích external entities, xác định process boundary, kiểm tra data flow consistency</t>
+  </si>
+  <si>
+    <t>Khi thiết kế Context Diagram cho Coworking Space Booking System, nhóm tranh luận: Notification System (SMS/Email) và Google OAuth có nên là External Entity riêng biệt hay gộp chung vào một entity "Third-party Services"?</t>
+  </si>
+  <si>
+    <t>Trong Context Diagram của hệ thống đặt chỗ coworking, Notification System (SMS/Email) và Google OAuth có nên tách thành 2 external entity riêng không, hay gộp chung thành "Third-party Services" cho gọn?</t>
+  </si>
+  <si>
+    <t>AI khuyến nghị tách thành 2 entity riêng biệt vì mỗi entity có data flow khác nhau hoàn toàn: Google OAuth nhận Authentication Request và trả về Token, còn Notification System chỉ nhận Notification Data một chiều. Gộp chung sẽ làm mờ data flow và vi phạm nguyên tắc Context Diagram: mỗi entity phải có data flow rõ ràng.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI đúng về nguyên tắc nhưng tôi nhận ra còn một lý do quan trọng hơn: nếu gộp chung, khi vẽ DFD-1 sau này sẽ không thể trace ngược lại được external entity nào xử lý luồng nào — vi phạm tính Traceability giữa các cấp DFD.
+Contextualization: Đề bài yêu cầu cụ thể "SMS or email" và "Google login" là 2 tính năng riêng biệt → phải thể hiện là 2 entity để khớp với requirement.
+Creative Synthesis: Quyết định dùng 6 External Entities: User, Space Manager, Admin, Payment Gateway, Notification System, Google OAuth. Mỗi entity có ít nhất 1 data flow vào và/hoặc ra hệ thống.
+Decision Ownership: Cấu trúc 6 entity này được giữ nhất quán từ Context Diagram xuống DFD-0 và DFD-1.</t>
+  </si>
+  <si>
+    <t>Picture evidence_for_entry5.png — Context Diagram final với 6 external entities, in folder week3/ GG Drive tại README.md
+Date: 26/05/2026</t>
+  </si>
+  <si>
+    <t>Khi vẽ data flow giữa Admin và hệ thống trong Context Diagram, tôi đặt luồng "Pending Availability List" từ System → Admin và "Approval Decision" từ Admin → System. Cần xác minh chiều mũi tên có đúng không.</t>
+  </si>
+  <si>
+    <t>Trong Context Diagram, data flow "Pending Availability List" nên đi từ System → Admin hay Admin → System? Và "Approval Decision" đi chiều nào?</t>
+  </si>
+  <si>
+    <t>AI xác nhận: "Pending Availability List" đi từ System → Admin (hệ thống đẩy danh sách chờ duyệt cho Admin xem). "Approval Decision" đi từ Admin → System (Admin gửi quyết định vào hệ thống). Đây là cặp request-response điển hình: System notify → Admin decide → System receive.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI xác nhận đúng. Tuy nhiên tôi phát hiện thêm một vấn đề AI không đề cập: trong đề bài, Space Manager "define availability" và Admin "approves" — nghĩa là phải có luồng từ Manager vào System trước, rồi System mới notify Admin. Context Diagram phải thể hiện đủ cả chuỗi này.
+Contextualization: Nếu bỏ sót luồng Manager → System → Admin thì Context Diagram thiếu business logic quan trọng: ai tạo ra dữ liệu trước khi Admin duyệt?
+Creative Synthesis: Bổ sung đầy đủ: Manager gửi "Space Availability Details" → System → System gửi "Pending List" → Admin → Admin gửi "Approval Decision" → System → System gửi "Approval Status" → Manager.
+Decision Ownership: Hoàn chỉnh tất cả data flows 2 chiều cho từng external entity trước khi nộp.</t>
+  </si>
+  <si>
+    <t>Khi hoàn thiện Context Diagram, tôi phân vân: Payment Gateway có cần nhận thêm luồng "Refund Request" từ System không, hay chỉ cần luồng "Payment Transaction Request" và "Transaction Status" là đủ?</t>
+  </si>
+  <si>
+    <t>Context Diagram cho Coworking Space có cần thêm data flow "Refund Request" từ System → Payment Gateway không? Hay chỉ cần 2 luồng cơ bản: Payment Transaction Request và Transaction Status?</t>
+  </si>
+  <si>
+    <t>AI gợi ý nên thêm "Refund Request" vào Context Diagram vì đề bài có nêu rõ "Cancellations made 12 hours prior are refundable" — đây là business requirement rõ ràng. Nếu không thể hiện ở Context Diagram thì sẽ thiếu traceability khi vẽ DFD.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI đúng về yêu cầu business. Nhưng tôi cần cân nhắc: Context Diagram vẽ ở mức RẤT CAO — chỉ thể hiện major data flows, không phải mọi sub-flow. Refund là một phần của payment flow, không nhất thiết phải là arrow riêng ở level Context.
+Contextualization: Nếu thêm quá nhiều data flow vào Context Diagram sẽ làm rối, mất đi tính tổng quan. Refund có thể gộp vào "Payment Transaction Request" với ghi chú, hoặc thể hiện rõ hơn ở DFD-1.
+Creative Synthesis: Quyết định KHÔNG thêm arrow riêng cho Refund ở Context Diagram. Thay vào đó đổi tên flow thành "Payment / Refund Request" để bao quát cả 2 trường hợp. DFD-1 sẽ tách chi tiết thành 2 sub-process.
+Decision Ownership: Nguyên tắc: Context Diagram chỉ thể hiện major flows, chi tiết hóa ở DFD-1 và DFD-2.</t>
+  </si>
+  <si>
+    <t>Khi thiết kế DFD-0 (Level 0), cần xác định hệ thống Coworking Space Booking có bao nhiêu Process chính. Nhóm đang tranh luận giữa 3 process hay 5 process.</t>
+  </si>
+  <si>
+    <t>DFD Level 0 của Coworking Space Booking System nên chia thành bao nhiêu process chính? Nhóm đang xem xét: (A) 3 process: Manage Booking, Manage Space, Manage Users. (B) 5 process: Search Space, Book Space, Process Payment, Manage Space Availability, Manage Users. Cách nào chuẩn hơn?</t>
+  </si>
+  <si>
+    <t>AI phân tích: cả 2 cách đều hợp lệ nhưng Option B (5 processes) chuẩn hơn cho DFD-0 vì mỗi process ánh xạ rõ ràng đến một nhóm external entity tương tác. Option A quá gộp, "Manage Booking" che giấu luồng Payment là một process quan trọng. AI khuyến nghị DFD-0 nên có 4-6 process để đủ chi tiết nhưng không quá phức tạp.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI phân tích đúng về số lượng process. Tuy nhiên tôi nhận thấy AI chưa xét tới yêu cầu đề bài về "verified users" và "encrypted communication" — đây là 2 concern liên quan đến Security/Authentication, cần có process riêng hoặc ít nhất là data store riêng.
+Contextualization: Đề bài nêu rõ "only verified users can access sensitive info" và "all communication is encrypted" → phải thể hiện được luồng authentication ở DFD level nào đó.
+Creative Synthesis: Quyết định DFD-0 có 5 process: (1) Manage Authentication, (2) Search &amp; Browse Spaces, (3) Manage Booking, (4) Process Payment &amp; Refund, (5) Manage Space Availability. Process 1 cover luồng Google OAuth và verified user.
+Decision Ownership: Cấu trúc 5 process này nhất quán với 6 external entities trong Context Diagram — mỗi entity tương tác với ít nhất 1 process.</t>
+  </si>
+  <si>
+    <t>Khi vẽ DFD-1 cho process "Manage Booking" (process 3 trong DFD-0), cần xác định data store nào cần thiết. Nhóm đang dùng 1 data store "Booking Database" cho tất cả, nhưng không chắc có nên tách thêm "Space Inventory" không.</t>
+  </si>
+  <si>
+    <t>Trong DFD-1 của process Manage Booking, có cần data store riêng cho "Space Inventory / Availability" không, hay dùng chung 1 data store "Booking DB" là đủ? Xét theo luồng: check availability → create booking → update space status.</t>
+  </si>
+  <si>
+    <t>AI giải thích: nên tách thành 2 data stores: (1) Booking Records — lưu thông tin đặt chỗ của khách, (2) Space Inventory — lưu trạng thái và lịch trống của từng không gian. Lý do: check availability đọc từ Space Inventory, create booking ghi vào Booking Records VÀ update Space Inventory. Nếu gộp chung thì data flow sẽ bị lộn xộn và không phản ánh đúng thực tế.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI đúng hoàn toàn. Tôi kiểm tra lại: nếu gộp 1 data store thì process "Check Availability" và process "Update Space Status" đều đọc/ghi vào cùng 1 nơi — sẽ không phân biệt được luồng nào đọc gì, ghi gì.
+Contextualization: Trong thực tế hệ thống coworking, Space Inventory phải được Space Manager cập nhật và Admin duyệt — đây là luồng hoàn toàn tách biệt với luồng đặt chỗ của Customer. Cần 2 data store riêng để thể hiện điều này.
+Creative Synthesis: Quyết định DFD-1 của Manage Booking sử dụng 3 data stores: D1-Booking Records, D2-Space Inventory, D3-User Accounts. Mỗi data store chỉ được truy cập bởi process có lý do nghiệp vụ rõ ràng.
+Decision Ownership: Nguyên tắc data store: tách theo đối tượng nghiệp vụ, không tách theo kỹ thuật hay gộp theo sự tiện lợi.</t>
+  </si>
+  <si>
+    <t>Khi hoàn thiện DFD-2 (Level 2) cho process "Process Payment &amp; Refund", nhóm cần quyết định: luồng "Cancellation / Refund" có nên tạo thành sub-process riêng trong DFD-2 không, hay để ở DFD-1 là đủ?</t>
+  </si>
+  <si>
+    <t>Trong DFD-2 của process "Process Payment &amp; Refund", có cần tách "Process Cancellation &amp; Refund" thành sub-process riêng không? Hay chỉ cần thể hiện ở DFD-1 là: Customer gửi Cancellation Request → System check 12h rule → System gửi Refund Request → Payment Gateway?</t>
+  </si>
+  <si>
+    <t>AI gợi ý: nếu business logic của refund đủ phức tạp (check điều kiện 12h, tính % hoàn tiền, cập nhật booking status, gửi notification) thì nên tách thành sub-process ở DFD-2. Nếu đơn giản thì DFD-1 là đủ. AI đề xuất DFD-2 cho "Process Cancellation" với các sub-process: (1) Validate Cancellation Request, (2) Calculate Refund Amount, (3) Send Refund to Gateway, (4) Update Booking Status.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI gợi ý 4 sub-processes khá chi tiết. Tôi đánh giá: với scope bài lab SWR302, decompose đến level 2 với 4 sub-process cho một feature là vừa đủ, không over-engineer. Tuy nhiên cần kiểm tra balance: các process khác ở DFD-2 có được decompose đến mức tương đương không?
+Contextualization: Đề bài nêu rõ điều kiện "12 hours prior" — đây là business rule cụ thể cần được thể hiện trong DFD như một decision point. Nếu bỏ qua thì DFD-2 không cover được requirement quan trọng này.
+Creative Synthesis: Quyết định DFD-2 của Process Payment có 4 sub-processes như AI gợi ý, nhưng bổ sung data flow từ D1-Booking Records vào step Validate (để check booking date và tính 12h). Đây là chi tiết AI bỏ sót.
+Decision Ownership: Nguyên tắc: chỉ vẽ DFD-2 cho process có business logic phức tạp (≥3 bước). Process đơn giản giữ ở DFD-1.</t>
+  </si>
+  <si>
+    <t>007</t>
+  </si>
+  <si>
+    <t>AI gợi ý chỉ cần 2 data flows cho Payment Gateway trong Context Diagram: "Payment Transaction Request" và "Transaction Status" là đủ, bỏ qua hoàn toàn luồng refund.</t>
+  </si>
+  <si>
+    <t>Đề bài nêu rõ "Cancellations made 12 hours prior are refundable" — đây là business requirement buộc phải có luồng refund giữa System và Payment Gateway. Chỉ 2 flow cơ bản là thiếu requirement.</t>
+  </si>
+  <si>
+    <t>Đọc lại đề bài requirement sau khi AI trả lời và so sánh từng external entity với business requirements được liệt kê.</t>
+  </si>
+  <si>
+    <t>Không tạo arrow Refund riêng ở Context Diagram (để giữ tổng quan) nhưng đổi label flow thành "Payment / Refund Request" và thể hiện chi tiết ở DFD-1. Ghi chú trong bài nộp.</t>
+  </si>
+  <si>
+    <t>009</t>
+  </si>
+  <si>
+    <t>AI gợi ý DFD-1 của Manage Booking chỉ cần 1 data store "Booking Database" gộp chung mọi thứ, cho rằng việc tách data store là "optional" và chỉ cần thiết khi hệ thống lớn.</t>
+  </si>
+  <si>
+    <t>Trong DFD, data store phải phản ánh đúng đối tượng nghiệp vụ, không phụ thuộc vào quy mô hệ thống. Space Inventory và Booking Records là 2 đối tượng khác nhau hoàn toàn — Space Manager cập nhật Space Inventory, còn Customer tạo Booking Records. Gộp chung vi phạm nguyên tắc DFD.</t>
+  </si>
+  <si>
+    <t>Phân tích actors: Space Manager không tương tác với Booking Records nhưng tương tác với Space Inventory → 2 entity nghiệp vụ khác nhau → phải là 2 data store.</t>
+  </si>
+  <si>
+    <t>Tách thành 3 data stores trong DFD-1: D1-Booking Records, D2-Space Inventory, D3-User Accounts. Kiểm tra lại từng data flow để đảm bảo đúng đối tượng.</t>
+  </si>
+  <si>
+    <t>Tại sao xóa Use Case Discount khỏi biểu đồ UML?</t>
+  </si>
+  <si>
+    <t>✅ AI gợi ý &lt;&lt;extend&gt;&gt; nhưng Discount là business rule, không phải UC</t>
+  </si>
+  <si>
+    <t>evidence_entry1.png</t>
+  </si>
+  <si>
+    <t>Tại sao Prepay không &lt;&lt;include&gt;&gt; Send Notification?</t>
+  </si>
+  <si>
+    <t>✅ Nếu SMS API sập, Payment vẫn phải thành công — chúng độc lập</t>
+  </si>
+  <si>
+    <t>evidence_entry2.png</t>
+  </si>
+  <si>
+    <t>Tại sao không dùng "Manage" làm tên Use Case?</t>
+  </si>
+  <si>
+    <t>✅ "Manage" mơ hồ, che giấu business rules, developer không biết code gì</t>
+  </si>
+  <si>
+    <t>evidence_entry3.png</t>
+  </si>
+  <si>
+    <t>004</t>
+  </si>
+  <si>
+    <t>Tại sao Space Manager không có tính năng Register public?</t>
+  </si>
+  <si>
+    <t>✅ Manager là nhân viên nội bộ B2C, không phải user vãng lai C2C</t>
+  </si>
+  <si>
+    <t>evidence_entry4.png</t>
+  </si>
+  <si>
+    <t>Tại sao label flow Payment Gateway thành "Payment/Refund Request"?</t>
+  </si>
+  <si>
+    <t>✅ AI bỏ sót refund requirement — phát hiện khi đọc lại đề bài</t>
+  </si>
+  <si>
+    <t>evidence_entry7.png</t>
+  </si>
+  <si>
+    <t>Tại sao DFD-1 cần 3 data stores thay vì 1?</t>
+  </si>
+  <si>
+    <t>✅ Space Inventory và Booking Records là 2 đối tượng nghiệp vụ khác nhau</t>
+  </si>
+  <si>
+    <t>evidence_entry9.png</t>
   </si>
 </sst>
 </file>
@@ -767,7 +969,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -851,8 +1053,42 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -877,8 +1113,24 @@
         <bgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F4F7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDE1E9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -901,11 +1153,26 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFAAAAAA"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFAAAAAA"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFAAAAAA"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFAAAAAA"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -942,20 +1209,53 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1271,7 +1571,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="19"/>
@@ -1327,7 +1627,7 @@
         <v>7</v>
       </c>
       <c r="C10">
-        <v>10</v>
+        <v>26</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1335,7 +1635,7 @@
         <v>8</v>
       </c>
       <c r="C11" s="3">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1343,7 +1643,7 @@
         <v>9</v>
       </c>
       <c r="C12" s="4">
-        <v>0.4</v>
+        <v>0.38400000000000001</v>
       </c>
       <c r="E12" s="5"/>
     </row>
@@ -1352,7 +1652,7 @@
         <v>10</v>
       </c>
       <c r="C13" s="3">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -1374,19 +1674,33 @@
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="7" t="s">
+    <row r="17" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A17" s="24" t="s">
         <v>125</v>
       </c>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
+      <c r="B17" s="24" t="s">
+        <v>126</v>
+      </c>
+      <c r="C17" s="24" t="s">
+        <v>127</v>
+      </c>
+      <c r="D17" s="24" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A18" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="B18" s="25" t="s">
+        <v>130</v>
+      </c>
+      <c r="C18" s="25" t="s">
+        <v>131</v>
+      </c>
+      <c r="D18" s="25" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="7"/>
@@ -1421,7 +1735,7 @@
         <v>20</v>
       </c>
       <c r="B24" s="8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C24" s="9"/>
     </row>
@@ -1430,7 +1744,7 @@
         <v>21</v>
       </c>
       <c r="B25" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C25" s="9"/>
     </row>
@@ -1439,7 +1753,7 @@
         <v>22</v>
       </c>
       <c r="B26" s="8">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C26" s="9"/>
     </row>
@@ -1448,7 +1762,7 @@
         <v>23</v>
       </c>
       <c r="B27" s="8">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C27" s="9"/>
     </row>
@@ -1475,7 +1789,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>24</v>
       </c>
       <c r="B1" s="19"/>
@@ -1487,7 +1801,7 @@
       <c r="H1" s="19"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="18" t="s">
         <v>25</v>
       </c>
       <c r="B2" s="19"/>
@@ -1629,64 +1943,150 @@
       </c>
     </row>
     <row r="8" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
-      <c r="H8" s="7"/>
+      <c r="A8" s="7">
+        <v>5</v>
+      </c>
+      <c r="B8" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="27" t="s">
+        <v>133</v>
+      </c>
+      <c r="E8" s="27" t="s">
+        <v>134</v>
+      </c>
+      <c r="F8" s="27" t="s">
+        <v>135</v>
+      </c>
+      <c r="G8" s="27" t="s">
+        <v>136</v>
+      </c>
+      <c r="H8" s="28" t="s">
+        <v>137</v>
+      </c>
     </row>
     <row r="9" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
-      <c r="H9" s="7"/>
+      <c r="A9" s="7">
+        <v>6</v>
+      </c>
+      <c r="B9" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C9" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="D9" s="27" t="s">
+        <v>138</v>
+      </c>
+      <c r="E9" s="27" t="s">
+        <v>139</v>
+      </c>
+      <c r="F9" s="27" t="s">
+        <v>140</v>
+      </c>
+      <c r="G9" s="27" t="s">
+        <v>141</v>
+      </c>
+      <c r="H9" s="28"/>
     </row>
     <row r="10" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
-      <c r="H10" s="7"/>
+      <c r="A10" s="7">
+        <v>7</v>
+      </c>
+      <c r="B10" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="C10" s="26" t="s">
+        <v>21</v>
+      </c>
+      <c r="D10" s="27" t="s">
+        <v>142</v>
+      </c>
+      <c r="E10" s="27" t="s">
+        <v>143</v>
+      </c>
+      <c r="F10" s="27" t="s">
+        <v>144</v>
+      </c>
+      <c r="G10" s="27" t="s">
+        <v>145</v>
+      </c>
+      <c r="H10" s="28"/>
     </row>
     <row r="11" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
-      <c r="H11" s="7"/>
+      <c r="A11" s="7">
+        <v>8</v>
+      </c>
+      <c r="B11" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C11" s="26" t="s">
+        <v>20</v>
+      </c>
+      <c r="D11" s="27" t="s">
+        <v>146</v>
+      </c>
+      <c r="E11" s="27" t="s">
+        <v>147</v>
+      </c>
+      <c r="F11" s="27" t="s">
+        <v>148</v>
+      </c>
+      <c r="G11" s="27" t="s">
+        <v>149</v>
+      </c>
+      <c r="H11" s="28"/>
     </row>
     <row r="12" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
+      <c r="A12" s="7">
+        <v>9</v>
+      </c>
+      <c r="B12" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C12" s="26" t="s">
+        <v>23</v>
+      </c>
+      <c r="D12" s="27" t="s">
+        <v>150</v>
+      </c>
+      <c r="E12" s="27" t="s">
+        <v>151</v>
+      </c>
+      <c r="F12" s="27" t="s">
+        <v>152</v>
+      </c>
+      <c r="G12" s="27" t="s">
+        <v>153</v>
+      </c>
+      <c r="H12" s="28"/>
     </row>
     <row r="13" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
-      <c r="H13" s="7"/>
+      <c r="A13" s="7">
+        <v>10</v>
+      </c>
+      <c r="B13" s="7" t="s">
+        <v>111</v>
+      </c>
+      <c r="C13" s="26" t="s">
+        <v>22</v>
+      </c>
+      <c r="D13" s="27" t="s">
+        <v>154</v>
+      </c>
+      <c r="E13" s="27" t="s">
+        <v>155</v>
+      </c>
+      <c r="F13" s="27" t="s">
+        <v>156</v>
+      </c>
+      <c r="G13" s="27" t="s">
+        <v>157</v>
+      </c>
+      <c r="H13" s="28"/>
     </row>
     <row r="14" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7"/>
@@ -1839,7 +2239,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="22" t="s">
         <v>39</v>
       </c>
       <c r="B1" s="19"/>
@@ -1849,7 +2249,7 @@
       <c r="F1" s="19"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="21" t="s">
         <v>40</v>
       </c>
       <c r="B2" s="19"/>
@@ -1879,20 +2279,44 @@
       </c>
     </row>
     <row r="4" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7"/>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" s="7"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
+      <c r="A4" s="30" t="s">
+        <v>158</v>
+      </c>
+      <c r="B4" s="29" t="s">
+        <v>54</v>
+      </c>
+      <c r="C4" s="30" t="s">
+        <v>159</v>
+      </c>
+      <c r="D4" s="30" t="s">
+        <v>160</v>
+      </c>
+      <c r="E4" s="30" t="s">
+        <v>161</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="105.6" x14ac:dyDescent="0.25">
+      <c r="A5" s="30" t="s">
+        <v>163</v>
+      </c>
+      <c r="B5" s="29" t="s">
+        <v>63</v>
+      </c>
+      <c r="C5" s="30" t="s">
+        <v>164</v>
+      </c>
+      <c r="D5" s="30" t="s">
+        <v>165</v>
+      </c>
+      <c r="E5" s="30" t="s">
+        <v>166</v>
+      </c>
+      <c r="F5" s="30" t="s">
+        <v>167</v>
+      </c>
     </row>
     <row r="6" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7"/>
@@ -2128,7 +2552,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D30"/>
+  <dimension ref="A1:D33"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2138,7 +2562,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="20" t="s">
         <v>66</v>
       </c>
       <c r="B1" s="19"/>
@@ -2146,7 +2570,7 @@
       <c r="D1" s="19"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="20" t="s">
+      <c r="A2" s="23" t="s">
         <v>67</v>
       </c>
       <c r="B2" s="19"/>
@@ -2179,7 +2603,7 @@
       <c r="B6" s="13" t="s">
         <v>74</v>
       </c>
-      <c r="C6" s="12" t="s">
+      <c r="C6" s="34" t="s">
         <v>75</v>
       </c>
       <c r="D6" s="13"/>
@@ -2191,7 +2615,7 @@
       <c r="B7" s="13" t="s">
         <v>77</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="34" t="s">
         <v>75</v>
       </c>
       <c r="D7" s="13"/>
@@ -2350,29 +2774,89 @@
         <v>98</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="9" t="s">
+    <row r="28" spans="1:4" ht="92.4" x14ac:dyDescent="0.25">
+      <c r="A28" s="31" t="s">
         <v>34</v>
       </c>
-      <c r="B28" s="7"/>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="9" t="s">
+      <c r="B28" s="32" t="s">
+        <v>168</v>
+      </c>
+      <c r="C28" s="32" t="s">
+        <v>169</v>
+      </c>
+      <c r="D28" s="33" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="105.6" x14ac:dyDescent="0.25">
+      <c r="A29" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="B29" s="7"/>
-      <c r="C29" s="7"/>
-      <c r="D29" s="7"/>
-    </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="9" t="s">
+      <c r="B29" s="32" t="s">
+        <v>171</v>
+      </c>
+      <c r="C29" s="32" t="s">
+        <v>172</v>
+      </c>
+      <c r="D29" s="33" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="118.8" x14ac:dyDescent="0.25">
+      <c r="A30" s="31" t="s">
         <v>37</v>
       </c>
-      <c r="B30" s="7"/>
-      <c r="C30" s="7"/>
-      <c r="D30" s="7"/>
+      <c r="B30" s="32" t="s">
+        <v>174</v>
+      </c>
+      <c r="C30" s="32" t="s">
+        <v>175</v>
+      </c>
+      <c r="D30" s="33" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="92.4" x14ac:dyDescent="0.25">
+      <c r="A31" s="31" t="s">
+        <v>177</v>
+      </c>
+      <c r="B31" s="32" t="s">
+        <v>178</v>
+      </c>
+      <c r="C31" s="32" t="s">
+        <v>179</v>
+      </c>
+      <c r="D31" s="33" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" ht="79.2" x14ac:dyDescent="0.25">
+      <c r="A32" s="31" t="s">
+        <v>158</v>
+      </c>
+      <c r="B32" s="32" t="s">
+        <v>181</v>
+      </c>
+      <c r="C32" s="32" t="s">
+        <v>182</v>
+      </c>
+      <c r="D32" s="33" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" ht="92.4" x14ac:dyDescent="0.25">
+      <c r="A33" s="31" t="s">
+        <v>163</v>
+      </c>
+      <c r="B33" s="32" t="s">
+        <v>184</v>
+      </c>
+      <c r="C33" s="32" t="s">
+        <v>185</v>
+      </c>
+      <c r="D33" s="33" t="s">
+        <v>186</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Upload Auditlog week 4 & 5
</commit_message>
<xml_diff>
--- a/SWR302_SE20A07_DE190512_MaiVanLuong.xlsx
+++ b/SWR302_SE20A07_DE190512_MaiVanLuong.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\SU26\SWR\auditlog\ai-audit-log-MaiLuong1906\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8439F8C0-8CD0-4FC0-B728-4D74B2D98661}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{344DBEC6-D497-40EA-8EF3-928BA397DAE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-14505" yWindow="0" windowWidth="14610" windowHeight="15585" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="1. Metadata &amp; Summary" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="225" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="269">
   <si>
     <t>AI AUDIT LOG - METADATA &amp; SUMMARY</t>
   </si>
@@ -961,6 +961,292 @@
   <si>
     <t>evidence_entry9.png</t>
   </si>
+  <si>
+    <t>Phân tích State Diagram, Swimlane Diagram, Data Dictionary, viết Method section paper</t>
+  </si>
+  <si>
+    <t>16 lần (tuần 4-5)</t>
+  </si>
+  <si>
+    <t>Phát hiện thiếu trạng thái UML, đồng bộ enum giữa SRS và Data Dictionary, cấu trúc paper Method</t>
+  </si>
+  <si>
+    <t>Khi vẽ State Diagram cho object Space Reservation, đề bài chỉ yêu cầu 6 trạng thái cơ bản: Requested → Paid → Confirmed → Used → Archived, và Confirmed → Cancelled → Refunded. Tôi muốn kiểm tra liệu 6 trạng thái này đã đủ để mô tả thực tế hệ thống thanh toán trực tuyến chưa.</t>
+  </si>
+  <si>
+    <t>Đề bài yêu cầu State Diagram cho Space Reservation với 6 trạng thái: Requested, Paid, Confirmed, Used, Archived, Cancelled, Refunded. Với một hệ thống prepay online thực tế (có cổng thanh toán), 6 trạng thái này có đủ để mô tả mọi tình huống không? Có thiếu trạng thái nào quan trọng không?</t>
+  </si>
+  <si>
+    <t>AI phân tích: 6 trạng thái của đề bài là "happy path" — chỉ mô tả luồng thành công. Trong thực tế, giữa Requested và Paid cần có trạng thái trung gian "Awaiting Payment" vì người dùng phải nhập thẻ và chờ phản hồi từ cổng thanh toán — đây không phải là chuyển đổi tức thì. Ngoài ra cần xử lý 2 trường hợp lỗi: thanh toán bị từ chối (Payment Failed) và quá hạn thanh toán (Expired) nếu user bỏ giữa chừng. AI cũng gợi ý thêm trạng thái Rescheduled vì đề bài có yêu cầu chức năng "reschedule" nhưng 6 trạng thái gốc không thể hiện điều này.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI phân tích đúng và phát hiện một gap quan trọng trong đề bài — đề bài liệt kê 6 trạng thái nhưng lại có yêu cầu chức năng "reschedule" ở phần mô tả nghiệp vụ (Customers can ... reschedule), nghĩa là 6 trạng thái gốc chưa đủ để cover toàn bộ functional requirements.
+Contextualization: Nếu chỉ vẽ đúng 6 trạng thái như đề bài, giám khảo sẽ hỏi: "Reschedule thì object chuyển sang state nào?" — nếu không có state đó thì State Diagram không complete đối với spec.
+Creative Synthesis: Quyết định mở rộng State Diagram thành 9 trạng thái: Requested → Awaiting Payment → Paid → Confirmed → Used → Archived (happy path); Awaiting Payment → Payment Failed → Awaiting Payment (retry loop); Awaiting Payment → Expired (timeout); Confirmed → Rescheduled → Confirmed (reschedule loop); Confirmed → Cancelled → Refunded.
+Decision Ownership: Giữ nguyên 6 trạng thái gốc làm "core path" nhưng bổ sung 3 trạng thái edge-case, có annotation rõ ràng trong báo cáo để giám khảo thấy nhóm hiểu đề bài là baseline tối thiểu, không phải toàn bộ.</t>
+  </si>
+  <si>
+    <t>Picture evidence_for_entry11.png — State Diagram final với 9 states (so với 6 states yêu cầu gốc), folder week4-5/ GG Drive tại README.md
+Date: 02/06/2026</t>
+  </si>
+  <si>
+    <t>Sau khi vẽ xong State Diagram với 9 trạng thái (entry 11), cần kiểm tra tính nhất quán: liệu transition "Payment timeout exceeded" từ Awaiting Payment → Expired có hợp lý về mặt UML không, vì Expired không có transition đi ra ngoài (dead-end state).</t>
+  </si>
+  <si>
+    <t>Trong State Diagram, trạng thái "Expired" (do payment timeout) chỉ có 1 transition đi vào, không có transition đi ra (không nối tới final state hoặc Archived). Đây có phải lỗi UML không? Nên xử lý thế nào?</t>
+  </si>
+  <si>
+    <t>AI xác nhận: đây là lỗi thiết kế thực sự — theo chuẩn UML, mọi state (trừ final state) phải có ít nhất 1 transition đi ra, nếu không sẽ tạo "deadlock state" — đối tượng bị mắc kẹt vĩnh viễn. AI gợi ý: Expired nên có transition trực tiếp tới Final State (kết thúc lifecycle của reservation đó), tương tự như nhánh Refunded → Final State.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI xác nhận đúng vấn đề kỹ thuật UML. Tuy nhiên tôi review thêm: nếu Expired đi thẳng tới Final State thì record reservation "biến mất" khỏi flow — nhưng trong thực tế, một booking bị expired vẫn cần lưu lại trong DB để audit (đã có trong bookings.booking_status enum: pending/confirmed/cancelled/used/archived — không có "expired"!).
+Contextualization: Tôi đối chiếu lại Data Dictionary tuần 5: booking_status chỉ có 5 giá trị (pending, confirmed, cancelled, used, archived), KHÔNG có "expired" hay "payment_failed". Đây là một inconsistency giữa State Diagram (9 states) và Database schema (5 status values) cần thống nhất.
+Creative Synthesis: Quyết định map các trạng thái tạm thời (Awaiting Payment, Payment Failed, Expired, Rescheduled) là "process states" chỉ tồn tại trong session/transaction, KHÔNG lưu permanent trong booking_status. Final mapping: Expired → booking_status="cancelled" khi lưu DB. Bổ sung Final State sau Expired trong State Diagram.
+Decision Ownership: Thêm 1 dòng vào Data Dictionary ghi chú: "State Diagram có process states (transient) khác với booking_status enum (persistent) — cần bảng mapping riêng".</t>
+  </si>
+  <si>
+    <t>Picture evidence_for_entry12.png — State Diagram sau khi thêm Final State cho nhánh Expired + bảng mapping State↔booking_status, folder week4-5/ GG Drive tại README.md
+Date: 02/06/2026</t>
+  </si>
+  <si>
+    <t>Khi vẽ Swimlane Diagram theo yêu cầu đề bài (Lanes: User, System, Manager, Admin — Activities: User searches→books→pays; System processes booking; Manager sets working hours; Admin approves), tôi thấy bài làm thực tế (Image 3) chỉ có 3 lanes: Customer, System, Payment Gateway — không có Manager và Admin. Cần quyết định có vẽ thêm 1 swimlane riêng cho Manager/Admin hay không.</t>
+  </si>
+  <si>
+    <t>Đề bài yêu cầu Swimlane Diagram có 4 lanes: User, System, Manager, Admin. Nhưng luồng "User searches → books → pays" chỉ liên quan đến User, System, Payment Gateway — không có Manager/Admin tham gia. Manager (set availability) và Admin (approve) là một luồng nghiệp vụ HOÀN TOÀN KHÁC. Có nên vẽ chung 1 Swimlane Diagram 4 lanes hay tách thành 2 diagram riêng?</t>
+  </si>
+  <si>
+    <t>AI khuyến nghị tách thành 2 Swimlane Diagram riêng biệt: Diagram 1 — "Booking &amp; Payment Flow" với lanes Customer/System/Payment Gateway (như Image 3 đã vẽ); Diagram 2 — "Availability Setup &amp; Approval Flow" với lanes Manager/System/Admin (tương ứng Luồng 3 trong Data Dictionary). AI giải thích: gộp 4 lanes vào 1 diagram sẽ tạo ra rất nhiều "empty cells" vì 2 nhóm actor không tương tác đồng thời trong cùng 1 use case — vi phạm nguyên tắc "mỗi Activity Diagram nên mô tả 1 business process hoàn chỉnh".</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI tư vấn hợp lý về mặt lý thuyết UML. Nhưng đề bài chỉ yêu cầu "Vẽ Swimlane Diagram" (số ít, 1 diagram) với 4 lanes named cụ thể — nếu tách thành 2 diagram, có nguy cơ giám khảo cho rằng nhóm không làm đúng đề bài literal.
+Contextualization: Tuy nhiên, mục tiêu thực sự của đề bài là kiểm tra hiểu biết về phân vai trò và luồng nghiệp vụ — không phải đếm số lượng diagram. Một Swimlane Diagram 4 lanes với 80% cells trống sẽ KHÔNG thể hiện được sự hiểu biết đó tốt như 2 diagram tập trung.
+Creative Synthesis: Quyết định làm 2 Swimlane Diagram riêng (đúng như Image 3 đã làm cho luồng Booking), kèm 1 đoạn giải thích ngắn trong báo cáo: "Đề bài yêu cầu 4 lanes nhưng nhóm nhận thấy 2 nhóm actor (Customer-facing vs Admin-facing) thuộc 2 business process độc lập, nên tách thành 2 diagram để tăng tính rõ ràng — đây là 2 sub-diagrams của tổng thể yêu cầu 4-lane".
+Decision Ownership: Diagram 1 (đã có - Image 3) cho luồng Booking &amp; Payment. Diagram 2 (Manager/System/Admin) cần vẽ bổ sung cho luồng Availability Setup &amp; Approval — tương ứng Luồng 3 trong Data Dictionary Processing Flows.</t>
+  </si>
+  <si>
+    <t>Picture evidence_for_entry13.png — Swimlane Diagram 1 (Customer/System/Payment Gateway, đã có) + Swimlane Diagram 2 (Manager/System/Admin, mới vẽ thêm), folder week4-5/ GG Drive tại README.md
+Date: 03/06/2026</t>
+  </si>
+  <si>
+    <t>Hoạt động nhóm tuần 4: dùng template Springer (Scopus Q4) trên Overleaf để viết phần Introduction, Related Work, Method, References cho paper. Nhóm cần tìm cách trình bày phần "Method" sao cho phản ánh đúng kiến trúc hệ thống Coworking Space đã thiết kế (Context Diagram, DFD, State Diagram) mà không bị trùng lặp với Chapter Design Specification trong SRS.</t>
+  </si>
+  <si>
+    <t>Khi viết phần "Method" của một paper Scopus Q4 dựa trên Springer template, cho một hệ thống Coworking Space Booking đã có Context Diagram, DFD, State Diagram trong SRS — nên trình bày Method section ở mức độ nào để không bị trùng lặp với SRS nhưng vẫn đủ chi tiết học thuật?</t>
+  </si>
+  <si>
+    <t>AI gợi ý cấu trúc Method section theo 3 tầng: (1) System Architecture Overview — tóm tắt Context Diagram ở mức conceptual, không lặp lại toàn bộ chi tiết SQL/DFD; (2) Core Workflow Description — mô tả lifecycle của Space Reservation bằng văn xuôi học thuật, tham chiếu đến State Diagram như Figure nhưng không liệt kê lại từng transition; (3) Key Design Decisions — phần SRS không có, đây là phần "đóng góp học thuật" giải thích TẠI SAO chọn thiết kế này (ví dụ: tại sao tách 2 swimlane riêng, tại sao có Awaiting Payment state). AI nhấn mạnh: paper Method section nên tập trung vào "rationale" (lý do thiết kế), còn SRS tập trung vào "specification" (đặc tả chi tiết).</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI phân biệt đúng vai trò của 2 loại tài liệu — đây là điểm tôi chưa nghĩ tới: SRS trả lời "WHAT", paper trả lời "WHY". Việc tận dụng lại các quyết định từ entry 11-13 (tại sao có Awaiting Payment, tại sao tách 2 swimlane) chính là "Key Design Decisions" — không cần research thêm, chỉ cần viết lại có học thuật.
+Contextualization: Paper Scopus Q4 thường yêu cầu Method section có "novelty" — không thể chỉ là báo cáo lại SRS. Phần rationale từ quá trình AI-assisted design chính là nguồn nội dung độc đáo cho Method section.
+Creative Synthesis: Cấu trúc Method section thành 3 subsection theo gợi ý AI, viết Key Design Decisions dựa trực tiếp trên 3 quyết định đã log ở entry 11, 12, 13 (mở rộng State Diagram, mapping state↔DB status, tách swimlane).
+Decision Ownership: Phân công: 1 thành viên viết Architecture Overview + Core Workflow (dựa trên diagram có sẵn), tôi viết Key Design Decisions (dựa trên AI audit log của chính mình).</t>
+  </si>
+  <si>
+    <t>Picture evidence_for_entry14.png — Outline 3-subsection của Method section trên Overleaf, folder week4-5/ GG Drive tại README.md
+Date: 03/06/2026</t>
+  </si>
+  <si>
+    <t>Khi tải template Springer Scopus Q4 từ trang Springer về Overleaf, nhóm gặp vấn đề: template có nhiều file .cls và .bst khác nhau (llncs, svjour3, sn-jnl...), cần xác định đúng template phù hợp với định dạng paper hội nghị/journal mà nhóm hướng tới.</t>
+  </si>
+  <si>
+    <t>Template Springer trên Overleaf có nhiều biến thể: llncs (Lecture Notes in Computer Science), svjour3, sn-jnl (Springer Nature journal). Với một paper về thiết kế hệ thống phần mềm (system design paper) dự định submit conference proceedings, template nào phù hợp nhất và cấu trúc section chuẩn là gì?</t>
+  </si>
+  <si>
+    <t>AI giải thích: llncs (Lecture Notes in Computer Science) phù hợp nhất cho conference proceedings về Computer Science, vì đây là format chuẩn cho các hội nghị thuộc Springer LNCS series — rất phổ biến cho paper sinh viên/early-career researcher. svjour3 và sn-jnl dùng cho journal article, có yêu cầu nghiêm ngặt hơn về structured abstract và declarations (funding, conflict of interest) không phù hợp với scope bài tập RBL. AI đề xuất cấu trúc: Title/Authors → Abstract → Introduction → Related Work → Method → Results/Discussion (nếu có) → Conclusion → References, dùng \bibliographystyle{splncs04}.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI đưa thông tin về các template variant khá chính xác về mặt khái niệm, nhưng tôi cần verify thực tế trên Overleaf vì các phiên bản template có thể đã được Springer cập nhật — tên file .cls/.bst chính xác có thể khác so với khi AI được train.
+Contextualization: Việc chọn sai template không chỉ là vấn đề hình thức — nếu dùng sai \bibliographystyle, References sẽ bị lỗi format hoặc không compile được trên Overleaf, ảnh hưởng đến deadline nộp.
+Creative Synthesis: Tôi tự vào Overleaf, tìm "Springer LNCS" trong gallery template, xác nhận tên file thực tế là llncs2track2_authors.tex và bibliographystyle splncs04 — khớp với gợi ý AI nên proceed.
+Decision Ownership: Chốt dùng llncs template, cấu trúc 7 section như AI gợi ý. Đây là quyết định mang tính hạ tầng (infrastructure decision) cho toàn bộ paper, ảnh hưởng đến mọi thành viên viết tiếp ở tuần 5.</t>
+  </si>
+  <si>
+    <t>Picture evidence_for_entry15.png — Screenshot Overleaf project với llncs template đã setup + compile thành công, folder week4-5/ GG Drive tại README.md
+Date: 03/06/2026</t>
+  </si>
+  <si>
+    <t>Khi thiết kế UI cho Space Detail (Image 1), giao diện hiển thị 4 mức giá: $7/giờ, $45/ngày, $250/tuần (-20%), $800/tháng (-30%). Cần xác định: 4 giá này nên lưu cứng trong database hay tính động từ giá theo giờ với hệ số giảm giá cố định?</t>
+  </si>
+  <si>
+    <t>UI hiển thị 4 mức giá cho 1 space: hourly $7, daily $45, weekly $250 (giảm 20%), monthly $800 (giảm 30%). Trong Data Dictionary, có nên lưu cả 4 giá trị (price_per_hour, price_per_day, price_per_week, price_per_month) trong bảng spaces, hay chỉ lưu price_per_hour và tính 3 giá còn lại bằng công thức với discount cố định 20%/30%?</t>
+  </si>
+  <si>
+    <t>AI phân tích 2 phương án: Phương án A (lưu cả 4 giá) cho phép Space Manager tùy chỉnh giá linh hoạt theo từng loại không gian (không phải mọi space đều giảm đúng 20%/30%). Phương án B (tính động) đảm bảo tính nhất quán toán học nhưng cứng hóa business rule, khó thay đổi discount theo từng campaign. AI khuyến nghị Phương án A vì linh hoạt hơn cho business thực tế, nhưng cần validation: weekly price phải &lt; hourly×24×7 và monthly price phải &lt; hourly×24×30.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI đúng về sự linh hoạt, và quan sát thực tế Data Dictionary tuần 5 ĐÃ chọn Phương án A (lưu riêng price_per_hour, price_per_day, price_per_week, price_per_month đều là field riêng trong bảng spaces) — quyết định này đã được đưa ra trước khi tôi hỏi AI, nhưng AI giúp xác nhận tính đúng đắn và bổ sung validation rule còn thiếu.
+Contextualization: Trường hợp thực tế: một space có thể có chương trình ưu đãi đặc biệt (ví dụ giảm 35% cho tháng đầu mở cửa) — nếu hardcode 20%/30% thì Manager không tự set được, phải sửa code.
+Creative Synthesis: Giữ nguyên 4 field riêng trong Data Dictionary (price_per_hour, price_per_day, price_per_week, price_per_month — đều "Giá trị &gt;= 0"), nhưng bổ sung thêm 1 cột "Constraint" ghi rõ: "price_per_week SHOULD be ≤ price_per_day × 7 × 0.8 (gợi ý), price_per_month SHOULD be ≤ price_per_day × 30 × 0.7" — là validation gợi ý (soft constraint), không phải hard CHECK constraint trong DB.
+Decision Ownership: Soft constraint cho phép Manager linh hoạt nhưng UI sẽ cảnh báo (warning, không block) nếu Manager đặt giá vô lý — quyết định UX này được note vào Group 2 Processing Flows.</t>
+  </si>
+  <si>
+    <t>Picture evidence_for_entry16.png — Data Dictionary Group 1, 4 dòng price_per_* với cột Constraint bổ sung soft-validation note, folder week4-5/ GG Drive tại README.md
+Date: 06/06/2026</t>
+  </si>
+  <si>
+    <t>Trong Data Dictionary Group 1, field "Card Number", "Card Expiry", "Card CVV" được ghi Database/Table = "UI Input" (không lưu DB) với chú thích "Không lưu trực tiếp dưới DB để bảo mật". Cần verify liệu cách ghi này có đủ rõ ràng về compliance (PCI-DSS) không, hay cần bổ sung thêm.</t>
+  </si>
+  <si>
+    <t>Trong Data Dictionary, 3 field Card Number/Expiry/CVV được đánh dấu "UI Input" và ghi chú "Không lưu trực tiếp dưới DB để bảo mật". Với một hệ thống thực tế xử lý thanh toán thẻ, ghi chú này có đủ để thể hiện compliance về bảo mật dữ liệu thẻ (PCI-DSS) không? Có thiếu thông tin quan trọng nào không?</t>
+  </si>
+  <si>
+    <t>AI giải thích: ghi chú "không lưu trực tiếp" là đúng hướng nhưng chưa đủ rõ về luồng dữ liệu thực tế đi đâu. Theo PCI-DSS, hệ thống KHÔNG được tự xử lý/lưu trữ raw card data — toàn bộ thông tin thẻ phải được gửi trực tiếp (tokenization) tới Payment Gateway (Stripe, VNPay...) qua iframe/SDK riêng, server của hệ thống chỉ nhận lại "payment token" hoặc "transaction reference". AI gợi ý bổ sung field "Payment Token" (lưu trong bookings) thay vì chỉ ghi "không lưu Card Number".</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI chỉ ra đúng gap quan trọng — Data Dictionary hiện tại có field "Payment Method" (enum: credit-card/e-wallet/bank-transfer) và "Total Price" trong bookings, nhưng KHÔNG có field nào lưu transaction reference/token để TRA SOÁT giao dịch sau này. Nếu khách hàng khiếu nại "tôi đã thanh toán nhưng không thấy confirm", hệ thống không có cách nào trace lại giao dịch với Payment Gateway.
+Contextualization: Đây liên quan trực tiếp đến UC Process Refund (đã thiết kế ở SWP391 tuần 3) — refund cần transaction_code để Payment Gateway xử lý hoàn tiền đúng giao dịch.
+Creative Synthesis: Bổ sung field mới vào Group 1: "Payment Transaction ID" — Database: bookings, Data Type: String(100), Description: "Mã giao dịch trả về từ Payment Gateway sau khi thanh toán thành công, dùng để tra soát/hoàn tiền", Constraint: "Nullable khi Payment Status = pending; Not Null khi = paid".
+Decision Ownership: Cập nhật Data Dictionary thêm 1 field mới — đây là field do AI gợi ý mà bài làm gốc chưa có, cần điền bổ sung trước khi nộp.</t>
+  </si>
+  <si>
+    <t>Picture evidence_for_entry17.png — Data Dictionary trước/sau khi thêm field "Payment Transaction ID", folder week4-5/ GG Drive tại README.md
+Date: 06/06/2026</t>
+  </si>
+  <si>
+    <t>Trong UI Space Detail (Image 1), tổng tiền "Tổng cộng $45" hiển thị ngay khi chọn "Theo ngày" mà chưa cần bấm "Tiếp tục đặt chỗ". Đối chiếu với Processing Flow Luồng 1 bước 4-5 trong Data Dictionary: "Chọn ngày thuê, thời lượng... bấm Tiếp tục đặt chỗ" → "Tự động tính tổng tiền". Có mâu thuẫn giữa UI thực tế và Processing Flow mô tả không?</t>
+  </si>
+  <si>
+    <t>UI (Image 1) hiển thị "Tổng cộng $45" ngay khi user thay đổi lựa chọn "Thời lượng" — tức tính real-time trên client. Nhưng Processing Flow trong Data Dictionary ghi: bước 4 (Actor chọn + bấm Tiếp tục) → bước 5 (System tự động tính tổng tiền). Vậy việc tính tổng tiền nên là client-side (real-time) hay server-side (sau khi submit)? Có cần làm cả 2?</t>
+  </si>
+  <si>
+    <t>AI giải thích: nên làm CẢ HAI nhưng với vai trò khác nhau. Client-side calculation (real-time khi đổi dropdown "Thời lượng") chỉ để hiển thị UX preview ngay lập tức — dùng công thức đơn giản (giá × hệ số giảm) chạy trong React state. Server-side calculation (khi bấm "Tiếp tục đặt chỗ", bước 5 trong flow) là tính toán CHÍNH THỨC, authoritative — vì giá có thể thay đổi giữa lúc user xem trang và lúc submit (Manager update giá), hoặc có thể có promotion code áp dụng thêm. AI nhấn mạnh: KHÔNG BAO GIỜ tin tưởng giá tính từ client khi tạo booking — total_price lưu vào DB phải là kết quả tính lại từ server.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI đưa ra nguyên tắc bảo mật quan trọng tương tự kiến thức đã áp dụng ở SWP391 entry 004 (total_price là snapshot, không tin client). Đây là một pattern lặp lại giữa 2 project — cho thấy nguyên tắc "never trust client-side calculation for financial data" là universal.
+Contextualization: Nếu chỉ tính client-side và submit total_price từ React state lên server, một user có kiến thức kỹ thuật có thể sửa request body để trả giá thấp hơn — lỗ hổng bảo mật nghiêm trọng (price manipulation).
+Creative Synthesis: Quyết định: UI hiển thị "Tổng cộng" real-time (client-side, cho UX) NHƯNG khi submit "Tiếp tục đặt chỗ", request chỉ gửi space_id + duration_type + hours_count (không gửi total_price), server tự tính lại total_price từ price_per_* trong DB. Processing Flow bước 5 ("System tự động tính toán tổng tiền") được hiểu là server-side authoritative calculation — UI hiển thị sớm chỉ là preview.
+Decision Ownership: Bổ sung ghi chú vào Processing Flow Luồng 1: "Bước 4 UI có thể hiển thị preview tổng tiền real-time, nhưng giá trị chính thức luôn được tính lại ở bước 5 (server-side), không nhận total_price từ client request."</t>
+  </si>
+  <si>
+    <t>Picture evidence_for_entry18.png — Processing Flow Luồng 1 với ghi chú bổ sung về client vs server calculation, folder week4-5/ GG Drive tại README.md
+Date: 07/06/2026</t>
+  </si>
+  <si>
+    <t>Hoạt động nhóm tuần 5: viết tiếp phần "Proposed Method" trong paper trên Overleaf, dựa trên các thiết kế đã hoàn thiện (State Diagram 9 states, Swimlane 2 diagrams, Data Dictionary). Cần xác định cách trình bày "Proposed Method" sao cho liên kết được 3 artifact này thành 1 narrative mạch lạc, không rời rạc.</t>
+  </si>
+  <si>
+    <t>Phần "Proposed Method" của paper cần trình bày 3 artifact: (1) State Diagram 9 states cho Space Reservation, (2) 2 Swimlane Diagrams (Booking flow và Approval flow), (3) Data Dictionary cho module Booking. Làm sao kết nối 3 artifact này thành 1 mạch văn logic, tránh viết 3 đoạn rời rạc "Hình X cho thấy..."?</t>
+  </si>
+  <si>
+    <t>AI gợi ý cấu trúc theo "lifecycle narrative": bắt đầu từ góc nhìn lifecycle của một Space Reservation (dùng State Diagram làm khung xương), mỗi transition trong State Diagram được giải thích BẰNG cách tham chiếu tới Swimlane Diagram tương ứng (ai thực hiện hành động gây ra transition) VÀ Data Dictionary (field nào bị thay đổi giá trị). Ví dụ: "Transition từ Confirmed sang Cancelled (State Diagram) được thực hiện qua hành động Hủy đặt chỗ trong Swimlane 1, cập nhật booking_status và payment_status trong Data Dictionary (Group 1)". Cách này biến 3 artifact thành 1 câu chuyện thống nhất.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI gợi ý "lifecycle narrative" là một cách kể chuyện hay, nhưng tôi nhận ra cần kiểm tra: liệu MỌI transition trong State Diagram 9 states đều có thể map tới 1 hành động trong Swimlane và 1 thay đổi field trong Data Dictionary không? Nếu có transition nào "orphan" (không map được) thì đó là dấu hiệu thiết kế chưa đồng bộ.
+Contextualization: Đây chính là cơ hội để kiểm tra lại toàn bộ 3 artifact một lần cuối trước khi nộp — paper writing trở thành một bước "integration test" cho thiết kế.
+Creative Synthesis: Lập 1 bảng mapping 3 cột: State Transition | Swimlane Action | Data Dictionary Field Changed. Phát hiện: transition "Awaiting Payment → Payment Failed → Awaiting Payment" (retry loop, entry 11) chưa có action tương ứng trong Swimlane 1 (Image 3 chỉ có nhánh "No" quay lại "Confirm and provide payment details" — đúng nhưng chưa label rõ là "retry"). Bổ sung label "Retry payment" vào arrow "No" trong Swimlane 1.
+Decision Ownership: Bảng mapping 3 cột này trở thành Table 1 trong paper Proposed Method section, đồng thời là bằng chứng cho việc 3 artifact được thiết kế đồng bộ — value rất cao cho cả paper và SRS.</t>
+  </si>
+  <si>
+    <t>Picture evidence_for_entry19.png — Bảng mapping State Transition × Swimlane Action × Data Dictionary Field, dùng làm Table 1 trong paper, folder week4-5/ GG Drive tại README.md
+Date: 09/06/2026</t>
+  </si>
+  <si>
+    <t>Hoạt động nhóm tuần 5 còn yêu cầu "Update SRS hoàn thiện phần UC, Screens Flow, Database Design". Khi đối chiếu lại SRS đã viết ở tuần 1-3 với các artifact mới (State Diagram, Data Dictionary), phát hiện SRS phần Database Design (Table Description, mục "bookings") liệt kê field "status (PENDING/CONFIRMED/REJECTED/CANCELLED)" — nhưng Data Dictionary tuần 5 lại dùng "Booking Status: pending, confirmed, cancelled, used, archived". Hai bảng enum khác nhau.</t>
+  </si>
+  <si>
+    <t>SRS Database Design (viết tuần 1-3) định nghĩa bookings.status có 4 giá trị: PENDING, CONFIRMED, REJECTED, CANCELLED (chữ hoa). Data Dictionary tuần 5 định nghĩa Booking Status có 5 giá trị: pending, confirmed, cancelled, used, archived (chữ thường). Đây có phải là 2 lần thiết kế độc lập gây mâu thuẫn không? Nên hợp nhất thế nào?</t>
+  </si>
+  <si>
+    <t>AI xác nhận đây là mâu thuẫn thực sự cần hợp nhất — không chỉ khác về case (HOA/thường) mà còn khác về SET giá trị: SRS có "REJECTED" (Data Dictionary không có), Data Dictionary có "used" và "archived" (SRS không có). AI phân tích nguồn gốc: SRS được viết SỚM (tuần 1-3) dựa trên Use Case tổng quát (Owner reject booking request); Data Dictionary được viết SAU (tuần 5) dựa trên State Diagram chi tiết hơn — phản ánh đúng lifecycle thực tế hơn nhưng thiếu trạng thái "rejected by owner". AI khuyến nghị hợp nhất thành 1 enum chuẩn duy nhất, dùng làm Single Source of Truth.</t>
+  </si>
+  <si>
+    <t>Critical Thinking: AI phân tích đúng nguồn gốc 2 lần thiết kế độc lập — đây chính là rủi ro "documentation drift" khi project kéo dài nhiều tuần và do nhiều thành viên cùng cập nhật các phần khác nhau mà không sync với nhau.
+Contextualization: Việc owner "reject" một booking request (trước khi Paid) là tình huống khác với "cancel" một booking đã Confirmed (có thể đã Paid). Gộp 2 khái niệm này vào 1 trạng thái sẽ làm mất thông tin về NGUYÊN NHÂN booking không thành công.
+Creative Synthesis: Quyết định enum chuẩn cuối cùng (lowercase, theo convention Data Dictionary mới hơn): pending, confirmed, rejected, cancelled, used, archived — 6 giá trị, gộp cả 2 nguồn. "rejected" = Owner/Admin từ chối trước khi Paid; "cancelled" = Customer hủy sau khi Confirmed. Cập nhật cả SRS Database Design (đổi case + bổ sung used/archived) và Data Dictionary (bổ sung rejected) để đồng bộ.
+Decision Ownership: Tạo 1 file CHANGELOG.md trong repo ghi lại quyết định hợp nhất enum này, kèm ngày cập nhật, để các thành viên khác biết và không tạo thêm phiên bản enum thứ 3 trong các tuần sau.</t>
+  </si>
+  <si>
+    <t>Picture evidence_for_entry20.png — So sánh SRS Database Design vs Data Dictionary trước/sau hợp nhất enum booking_status (6 giá trị), CHANGELOG.md, folder week4-5/ GG Drive tại README.md
+Date: 09/06/2026</t>
+  </si>
+  <si>
+    <t>012</t>
+  </si>
+  <si>
+    <t>AI gợi ý State "Expired" (do payment timeout) nên có transition trực tiếp tới Final State để tuân thủ UML — không phân tích thêm việc trạng thái này cần được ánh xạ thế nào sang booking_status trong database.</t>
+  </si>
+  <si>
+    <t>Database booking_status enum (theo SRS gốc) không có giá trị "expired" hoặc tương đương. Nếu Expired đi thẳng Final State mà không map vào DB, hệ thống sẽ mất dữ liệu audit về các booking bị timeout — vi phạm yêu cầu traceability.</t>
+  </si>
+  <si>
+    <t>Đối chiếu State Diagram 9-state mới với Data Dictionary Group 1 (Booking Status enum) — phát hiện 4 process states (Awaiting Payment, Payment Failed, Expired, Rescheduled) không có trong enum 5 giá trị persistent.</t>
+  </si>
+  <si>
+    <t>Tạo bảng mapping State Diagram (process states, transient) ↔ booking_status (persistent enum). Expired → lưu DB là "cancelled" kèm metadata note "reason: payment_timeout".</t>
+  </si>
+  <si>
+    <t>020</t>
+  </si>
+  <si>
+    <t>AI ban đầu chỉ tập trung giải thích nguồn gốc khác nhau giữa SRS (PENDING/CONFIRMED/REJECTED/CANCELLED) và Data Dictionary (pending/confirmed/cancelled/used/archived), nhưng không tự nhận ra rằng đây là phiên bản SRS đã LỖI THỜI từ tuần 1-3, trong khi Data Dictionary tuần 5 mới hơn và sát thực tế hơn.</t>
+  </si>
+  <si>
+    <t>SRS Database Design viết ở tuần 1-3 chưa có State Diagram (chỉ có ở tuần 4) — enum trong SRS là phiên bản early-draft chưa qua kiểm chứng với lifecycle thực tế. Data Dictionary tuần 5 được thiết kế SAU State Diagram nên phản ánh đúng hơn, nhưng lại thiếu "rejected" — một trạng thái hợp lệ mà SRS có.</t>
+  </si>
+  <si>
+    <t>So sánh timeline tạo tài liệu: SRS Database Design (tuần 1-3, trước State Diagram) vs Data Dictionary (tuần 5, sau State Diagram) — nhận ra "outdated" không có nghĩa là sai hoàn toàn, mỗi tài liệu có insight riêng cần hợp nhất.</t>
+  </si>
+  <si>
+    <t>Hợp nhất thành enum chuẩn 6 giá trị: pending, confirmed, rejected, cancelled, used, archived. Tạo CHANGELOG.md ghi version enum mới + lý do, tránh tài liệu nào "thắng" tài liệu khác mà không có rationale.</t>
+  </si>
+  <si>
+    <t>20 entries (tuần 1-2:4, tuần 3:6, tuần 4:5, tuần 5:5)</t>
+  </si>
+  <si>
+    <t>Decomposition:6 | Pattern:4 | Abstraction:6 | Algorithms:4</t>
+  </si>
+  <si>
+    <t>4 cases (007,009 tuần3 | 012 tuần4 | 020 tuần5) — Lab ≥1/tuần ✅</t>
+  </si>
+  <si>
+    <t>20/20 entries = 100% có evidence path</t>
+  </si>
+  <si>
+    <t>011</t>
+  </si>
+  <si>
+    <t>Tại sao State Diagram có 9 states thay vì 6 như đề bài?</t>
+  </si>
+  <si>
+    <t>✅ Đề bài chỉ mô tả happy path, thiếu Awaiting Payment/Failed/Expired/Rescheduled</t>
+  </si>
+  <si>
+    <t>evidence_entry11.png</t>
+  </si>
+  <si>
+    <t>013</t>
+  </si>
+  <si>
+    <t>Tại sao tách Swimlane thành 2 diagram thay vì 1 diagram 4 lanes?</t>
+  </si>
+  <si>
+    <t>✅ 2 nhóm actor thuộc 2 business process độc lập, gộp sẽ tạo nhiều cell trống</t>
+  </si>
+  <si>
+    <t>evidence_entry13.png</t>
+  </si>
+  <si>
+    <t>017</t>
+  </si>
+  <si>
+    <t>Tại sao thêm field "Payment Transaction ID" vào Data Dictionary?</t>
+  </si>
+  <si>
+    <t>✅ Cần để tra soát/hoàn tiền — PCI-DSS yêu cầu tokenization, không lưu raw card data</t>
+  </si>
+  <si>
+    <t>evidence_entry17.png</t>
+  </si>
+  <si>
+    <t>Tại sao booking_status có 6 giá trị thay vì 4 (SRS) hoặc 5 (Data Dictionary)?</t>
+  </si>
+  <si>
+    <t>✅ Hợp nhất 2 phiên bản: SRS có "rejected", Data Dictionary có "used/archived" — gộp cả 2</t>
+  </si>
+  <si>
+    <t>evidence_entry20.png</t>
+  </si>
 </sst>
 </file>
 
@@ -969,7 +1255,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="29" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1031,22 +1317,6 @@
     </font>
     <font>
       <b/>
-      <sz val="12"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <i/>
-      <sz val="10"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
@@ -1084,6 +1354,84 @@
     <font>
       <i/>
       <sz val="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF555555"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="16"/>
+      <color rgb="FF2E75B6"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF2E75B6"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF666666"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF1E8449"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -1172,11 +1520,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1185,29 +1532,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -1222,40 +1572,102 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1571,14 +1983,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="3" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
@@ -1626,33 +2038,33 @@
       <c r="A10" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C10">
-        <v>26</v>
+      <c r="C10" s="21">
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="3">
-        <v>10</v>
+      <c r="C11" s="22">
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C12" s="4">
-        <v>0.38400000000000001</v>
-      </c>
-      <c r="E12" s="5"/>
+      <c r="C12" s="3">
+        <v>0.47599999999999998</v>
+      </c>
+      <c r="E12" s="4"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C13" s="3">
-        <v>2</v>
+      <c r="C13" s="23">
+        <v>4</v>
       </c>
     </row>
     <row r="15" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
@@ -1661,58 +2073,66 @@
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" s="6" t="s">
+      <c r="A16" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="B16" s="6" t="s">
+      <c r="B16" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="C16" s="6" t="s">
+      <c r="C16" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="D16" s="6" t="s">
+      <c r="D16" s="5" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="17" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
-      <c r="A17" s="24" t="s">
+      <c r="A17" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="B17" s="24" t="s">
+      <c r="B17" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="C17" s="24" t="s">
+      <c r="C17" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="D17" s="24" t="s">
+      <c r="D17" s="9" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
-      <c r="A18" s="25" t="s">
+      <c r="A18" s="10" t="s">
         <v>129</v>
       </c>
-      <c r="B18" s="25" t="s">
+      <c r="B18" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="C18" s="25" t="s">
+      <c r="C18" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="D18" s="25" t="s">
+      <c r="D18" s="10" t="s">
         <v>132</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A19" s="7"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
+    <row r="19" spans="1:4" ht="39.6" x14ac:dyDescent="0.25">
+      <c r="A19" s="24" t="s">
+        <v>129</v>
+      </c>
+      <c r="B19" s="24" t="s">
+        <v>187</v>
+      </c>
+      <c r="C19" s="25" t="s">
+        <v>188</v>
+      </c>
+      <c r="D19" s="24" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
+      <c r="A20" s="6"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
     </row>
     <row r="22" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
@@ -1720,51 +2140,51 @@
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="6" t="s">
+      <c r="A23" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="B23" s="6" t="s">
+      <c r="B23" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="5" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="7" t="s">
+      <c r="A24" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="B24" s="8">
-        <v>3</v>
-      </c>
-      <c r="C24" s="9"/>
+      <c r="B24" s="26">
+        <v>6</v>
+      </c>
+      <c r="C24" s="7"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="7" t="s">
+      <c r="A25" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="B25" s="8">
-        <v>2</v>
-      </c>
-      <c r="C25" s="9"/>
+      <c r="B25" s="26">
+        <v>4</v>
+      </c>
+      <c r="C25" s="7"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="7" t="s">
+      <c r="A26" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B26" s="8">
-        <v>3</v>
-      </c>
-      <c r="C26" s="9"/>
+      <c r="B26" s="26">
+        <v>6</v>
+      </c>
+      <c r="C26" s="7"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="7" t="s">
+      <c r="A27" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="B27" s="8">
-        <v>2</v>
-      </c>
-      <c r="C27" s="9"/>
+      <c r="B27" s="26">
+        <v>4</v>
+      </c>
+      <c r="C27" s="7"/>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -1789,434 +2209,594 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="18" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="18" t="s">
+      <c r="A2" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
     </row>
     <row r="3" spans="1:8" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>29</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="H3" s="6" t="s">
+      <c r="H3" s="5" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="100.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="7">
+      <c r="A4" s="6">
         <v>1</v>
       </c>
-      <c r="B4" s="7" t="s">
+      <c r="B4" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C4" s="7" t="s">
+      <c r="C4" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D4" s="7" t="s">
+      <c r="D4" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="E4" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="F4" s="7" t="s">
+      <c r="F4" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="H4" s="7" t="s">
+      <c r="H4" s="6" t="s">
         <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="100.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="7">
+      <c r="A5" s="6">
         <v>2</v>
       </c>
-      <c r="B5" s="7" t="s">
+      <c r="B5" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="D5" s="7" t="s">
+      <c r="D5" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="E5" s="6" t="s">
         <v>108</v>
       </c>
-      <c r="F5" s="7" t="s">
+      <c r="F5" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="6" t="s">
         <v>110</v>
       </c>
-      <c r="H5" s="7" t="s">
+      <c r="H5" s="6" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="100.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7">
+      <c r="A6" s="6">
         <v>3</v>
       </c>
-      <c r="B6" s="7" t="s">
+      <c r="B6" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="C6" s="7" t="s">
+      <c r="C6" s="6" t="s">
         <v>21</v>
       </c>
-      <c r="D6" s="7" t="s">
+      <c r="D6" s="6" t="s">
         <v>112</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="E6" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="F6" s="7" t="s">
+      <c r="F6" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="H6" s="7" t="s">
+      <c r="H6" s="6" t="s">
         <v>123</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7">
+      <c r="A7" s="6">
         <v>4</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="B7" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="C7" s="6" t="s">
         <v>116</v>
       </c>
-      <c r="D7" s="7" t="s">
+      <c r="D7" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="E7" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="F7" s="7" t="s">
+      <c r="F7" s="6" t="s">
         <v>119</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="H7" s="7" t="s">
+      <c r="H7" s="6" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7">
+      <c r="A8" s="6">
         <v>5</v>
       </c>
-      <c r="B8" s="7" t="s">
+      <c r="B8" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C8" s="26" t="s">
+      <c r="C8" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="27" t="s">
+      <c r="D8" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="E8" s="27" t="s">
+      <c r="E8" s="12" t="s">
         <v>134</v>
       </c>
-      <c r="F8" s="27" t="s">
+      <c r="F8" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="G8" s="27" t="s">
+      <c r="G8" s="12" t="s">
         <v>136</v>
       </c>
-      <c r="H8" s="28" t="s">
+      <c r="H8" s="13" t="s">
         <v>137</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="7">
+      <c r="A9" s="6">
         <v>6</v>
       </c>
-      <c r="B9" s="7" t="s">
+      <c r="B9" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C9" s="26" t="s">
+      <c r="C9" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="27" t="s">
+      <c r="D9" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="E9" s="27" t="s">
+      <c r="E9" s="12" t="s">
         <v>139</v>
       </c>
-      <c r="F9" s="27" t="s">
+      <c r="F9" s="12" t="s">
         <v>140</v>
       </c>
-      <c r="G9" s="27" t="s">
+      <c r="G9" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="H9" s="28"/>
+      <c r="H9" s="13"/>
     </row>
     <row r="10" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="7">
+      <c r="A10" s="6">
         <v>7</v>
       </c>
-      <c r="B10" s="7" t="s">
+      <c r="B10" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="C10" s="26" t="s">
+      <c r="C10" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="27" t="s">
+      <c r="D10" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="E10" s="27" t="s">
+      <c r="E10" s="12" t="s">
         <v>143</v>
       </c>
-      <c r="F10" s="27" t="s">
+      <c r="F10" s="12" t="s">
         <v>144</v>
       </c>
-      <c r="G10" s="27" t="s">
+      <c r="G10" s="12" t="s">
         <v>145</v>
       </c>
-      <c r="H10" s="28"/>
+      <c r="H10" s="13"/>
     </row>
     <row r="11" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="7">
+      <c r="A11" s="6">
         <v>8</v>
       </c>
-      <c r="B11" s="7" t="s">
+      <c r="B11" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="C11" s="26" t="s">
+      <c r="C11" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="27" t="s">
+      <c r="D11" s="12" t="s">
         <v>146</v>
       </c>
-      <c r="E11" s="27" t="s">
+      <c r="E11" s="12" t="s">
         <v>147</v>
       </c>
-      <c r="F11" s="27" t="s">
+      <c r="F11" s="12" t="s">
         <v>148</v>
       </c>
-      <c r="G11" s="27" t="s">
+      <c r="G11" s="12" t="s">
         <v>149</v>
       </c>
-      <c r="H11" s="28"/>
+      <c r="H11" s="13"/>
     </row>
     <row r="12" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="7">
+      <c r="A12" s="6">
         <v>9</v>
       </c>
-      <c r="B12" s="7" t="s">
+      <c r="B12" s="6" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="26" t="s">
+      <c r="C12" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="D12" s="27" t="s">
+      <c r="D12" s="12" t="s">
         <v>150</v>
       </c>
-      <c r="E12" s="27" t="s">
+      <c r="E12" s="12" t="s">
         <v>151</v>
       </c>
-      <c r="F12" s="27" t="s">
+      <c r="F12" s="12" t="s">
         <v>152</v>
       </c>
-      <c r="G12" s="27" t="s">
+      <c r="G12" s="12" t="s">
         <v>153</v>
       </c>
-      <c r="H12" s="28"/>
+      <c r="H12" s="13"/>
     </row>
     <row r="13" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="7">
+      <c r="A13" s="6">
         <v>10</v>
       </c>
-      <c r="B13" s="7" t="s">
+      <c r="B13" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="C13" s="26" t="s">
+      <c r="C13" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="D13" s="27" t="s">
+      <c r="D13" s="12" t="s">
         <v>154</v>
       </c>
-      <c r="E13" s="27" t="s">
+      <c r="E13" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="F13" s="27" t="s">
+      <c r="F13" s="12" t="s">
         <v>156</v>
       </c>
-      <c r="G13" s="27" t="s">
+      <c r="G13" s="12" t="s">
         <v>157</v>
       </c>
-      <c r="H13" s="28"/>
+      <c r="H13" s="13"/>
     </row>
     <row r="14" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
-      <c r="H14" s="7"/>
+      <c r="A14" s="6">
+        <v>11</v>
+      </c>
+      <c r="B14" s="33" t="s">
+        <v>36</v>
+      </c>
+      <c r="C14" s="27" t="s">
+        <v>20</v>
+      </c>
+      <c r="D14" s="28" t="s">
+        <v>190</v>
+      </c>
+      <c r="E14" s="28" t="s">
+        <v>191</v>
+      </c>
+      <c r="F14" s="28" t="s">
+        <v>192</v>
+      </c>
+      <c r="G14" s="28" t="s">
+        <v>193</v>
+      </c>
+      <c r="H14" s="29" t="s">
+        <v>194</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="7"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="7"/>
+      <c r="A15" s="6">
+        <v>12</v>
+      </c>
+      <c r="B15" s="33" t="s">
+        <v>38</v>
+      </c>
+      <c r="C15" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="D15" s="28" t="s">
+        <v>195</v>
+      </c>
+      <c r="E15" s="28" t="s">
+        <v>196</v>
+      </c>
+      <c r="F15" s="28" t="s">
+        <v>197</v>
+      </c>
+      <c r="G15" s="28" t="s">
+        <v>198</v>
+      </c>
+      <c r="H15" s="29" t="s">
+        <v>199</v>
+      </c>
     </row>
     <row r="16" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
-      <c r="H16" s="7"/>
+      <c r="A16" s="6">
+        <v>13</v>
+      </c>
+      <c r="B16" s="33" t="s">
+        <v>111</v>
+      </c>
+      <c r="C16" s="27" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" s="28" t="s">
+        <v>200</v>
+      </c>
+      <c r="E16" s="28" t="s">
+        <v>201</v>
+      </c>
+      <c r="F16" s="28" t="s">
+        <v>202</v>
+      </c>
+      <c r="G16" s="28" t="s">
+        <v>203</v>
+      </c>
+      <c r="H16" s="29" t="s">
+        <v>204</v>
+      </c>
     </row>
     <row r="17" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
-      <c r="H17" s="7"/>
+      <c r="A17" s="6">
+        <v>14</v>
+      </c>
+      <c r="B17" s="33" t="s">
+        <v>36</v>
+      </c>
+      <c r="C17" s="42" t="s">
+        <v>23</v>
+      </c>
+      <c r="D17" s="43" t="s">
+        <v>205</v>
+      </c>
+      <c r="E17" s="43" t="s">
+        <v>206</v>
+      </c>
+      <c r="F17" s="43" t="s">
+        <v>207</v>
+      </c>
+      <c r="G17" s="43" t="s">
+        <v>208</v>
+      </c>
+      <c r="H17" s="29" t="s">
+        <v>209</v>
+      </c>
     </row>
     <row r="18" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
-      <c r="H18" s="7"/>
+      <c r="A18" s="6">
+        <v>15</v>
+      </c>
+      <c r="B18" s="33" t="s">
+        <v>38</v>
+      </c>
+      <c r="C18" s="42" t="s">
+        <v>20</v>
+      </c>
+      <c r="D18" s="43" t="s">
+        <v>210</v>
+      </c>
+      <c r="E18" s="43" t="s">
+        <v>211</v>
+      </c>
+      <c r="F18" s="43" t="s">
+        <v>212</v>
+      </c>
+      <c r="G18" s="43" t="s">
+        <v>213</v>
+      </c>
+      <c r="H18" s="29" t="s">
+        <v>214</v>
+      </c>
     </row>
     <row r="19" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="7"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="7"/>
+      <c r="A19" s="6">
+        <v>16</v>
+      </c>
+      <c r="B19" s="33" t="s">
+        <v>36</v>
+      </c>
+      <c r="C19" s="42" t="s">
+        <v>22</v>
+      </c>
+      <c r="D19" s="43" t="s">
+        <v>215</v>
+      </c>
+      <c r="E19" s="43" t="s">
+        <v>216</v>
+      </c>
+      <c r="F19" s="43" t="s">
+        <v>217</v>
+      </c>
+      <c r="G19" s="43" t="s">
+        <v>218</v>
+      </c>
+      <c r="H19" s="29" t="s">
+        <v>219</v>
+      </c>
     </row>
     <row r="20" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
-      <c r="H20" s="7"/>
+      <c r="A20" s="6">
+        <v>17</v>
+      </c>
+      <c r="B20" s="33" t="s">
+        <v>38</v>
+      </c>
+      <c r="C20" s="42" t="s">
+        <v>21</v>
+      </c>
+      <c r="D20" s="43" t="s">
+        <v>220</v>
+      </c>
+      <c r="E20" s="43" t="s">
+        <v>221</v>
+      </c>
+      <c r="F20" s="43" t="s">
+        <v>222</v>
+      </c>
+      <c r="G20" s="43" t="s">
+        <v>223</v>
+      </c>
+      <c r="H20" s="29" t="s">
+        <v>224</v>
+      </c>
     </row>
     <row r="21" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="7"/>
-      <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
-      <c r="H21" s="7"/>
+      <c r="A21" s="6">
+        <v>18</v>
+      </c>
+      <c r="B21" s="33" t="s">
+        <v>111</v>
+      </c>
+      <c r="C21" s="42" t="s">
+        <v>23</v>
+      </c>
+      <c r="D21" s="43" t="s">
+        <v>225</v>
+      </c>
+      <c r="E21" s="43" t="s">
+        <v>226</v>
+      </c>
+      <c r="F21" s="43" t="s">
+        <v>227</v>
+      </c>
+      <c r="G21" s="43" t="s">
+        <v>228</v>
+      </c>
+      <c r="H21" s="29" t="s">
+        <v>229</v>
+      </c>
     </row>
     <row r="22" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="7"/>
-      <c r="B22" s="7"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
-      <c r="H22" s="7"/>
+      <c r="A22" s="6">
+        <v>19</v>
+      </c>
+      <c r="B22" s="33" t="s">
+        <v>36</v>
+      </c>
+      <c r="C22" s="42" t="s">
+        <v>20</v>
+      </c>
+      <c r="D22" s="43" t="s">
+        <v>230</v>
+      </c>
+      <c r="E22" s="43" t="s">
+        <v>231</v>
+      </c>
+      <c r="F22" s="43" t="s">
+        <v>232</v>
+      </c>
+      <c r="G22" s="43" t="s">
+        <v>233</v>
+      </c>
+      <c r="H22" s="29" t="s">
+        <v>234</v>
+      </c>
     </row>
     <row r="23" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="7"/>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
-      <c r="H23" s="7"/>
+      <c r="A23" s="6">
+        <v>20</v>
+      </c>
+      <c r="B23" s="33" t="s">
+        <v>38</v>
+      </c>
+      <c r="C23" s="42" t="s">
+        <v>22</v>
+      </c>
+      <c r="D23" s="43" t="s">
+        <v>235</v>
+      </c>
+      <c r="E23" s="43" t="s">
+        <v>236</v>
+      </c>
+      <c r="F23" s="43" t="s">
+        <v>237</v>
+      </c>
+      <c r="G23" s="43" t="s">
+        <v>238</v>
+      </c>
+      <c r="H23" s="29" t="s">
+        <v>239</v>
+      </c>
     </row>
     <row r="24" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="7"/>
-      <c r="B24" s="7"/>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
-      <c r="F24" s="7"/>
-      <c r="G24" s="7"/>
-      <c r="H24" s="7"/>
+      <c r="A24" s="6"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
+      <c r="G24" s="6"/>
+      <c r="H24" s="6"/>
     </row>
     <row r="25" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="7"/>
-      <c r="B25" s="7"/>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
-      <c r="G25" s="7"/>
-      <c r="H25" s="7"/>
+      <c r="A25" s="6"/>
+      <c r="B25" s="6"/>
+      <c r="C25" s="6"/>
+      <c r="D25" s="6"/>
+      <c r="E25" s="6"/>
+      <c r="F25" s="6"/>
+      <c r="G25" s="6"/>
+      <c r="H25" s="6"/>
     </row>
     <row r="26" spans="1:8" ht="79.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="7"/>
-      <c r="B26" s="7"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
-      <c r="H26" s="7"/>
+      <c r="A26" s="6"/>
+      <c r="B26" s="6"/>
+      <c r="C26" s="6"/>
+      <c r="D26" s="6"/>
+      <c r="E26" s="6"/>
+      <c r="F26" s="6"/>
+      <c r="G26" s="6"/>
+      <c r="H26" s="6"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2239,236 +2819,260 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="22" t="s">
+      <c r="A1" s="20" t="s">
         <v>39</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="19" t="s">
         <v>40</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
     </row>
     <row r="3" spans="1:6" ht="40.049999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
+      <c r="A3" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="5" t="s">
         <v>44</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="F3" s="6" t="s">
+      <c r="F3" s="5" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="4" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="30" t="s">
+      <c r="A4" s="15" t="s">
         <v>158</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="C4" s="30" t="s">
+      <c r="C4" s="15" t="s">
         <v>159</v>
       </c>
-      <c r="D4" s="30" t="s">
+      <c r="D4" s="15" t="s">
         <v>160</v>
       </c>
-      <c r="E4" s="30" t="s">
+      <c r="E4" s="15" t="s">
         <v>161</v>
       </c>
-      <c r="F4" s="30" t="s">
+      <c r="F4" s="15" t="s">
         <v>162</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="105.6" x14ac:dyDescent="0.25">
-      <c r="A5" s="30" t="s">
+      <c r="A5" s="15" t="s">
         <v>163</v>
       </c>
-      <c r="B5" s="29" t="s">
+      <c r="B5" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="C5" s="30" t="s">
+      <c r="C5" s="15" t="s">
         <v>164</v>
       </c>
-      <c r="D5" s="30" t="s">
+      <c r="D5" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="E5" s="30" t="s">
+      <c r="E5" s="15" t="s">
         <v>166</v>
       </c>
-      <c r="F5" s="30" t="s">
+      <c r="F5" s="15" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="6" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
+      <c r="A6" s="55" t="s">
+        <v>240</v>
+      </c>
+      <c r="B6" s="56" t="s">
+        <v>57</v>
+      </c>
+      <c r="C6" s="55" t="s">
+        <v>241</v>
+      </c>
+      <c r="D6" s="55" t="s">
+        <v>242</v>
+      </c>
+      <c r="E6" s="55" t="s">
+        <v>243</v>
+      </c>
+      <c r="F6" s="55" t="s">
+        <v>244</v>
+      </c>
     </row>
     <row r="7" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
+      <c r="A7" s="55" t="s">
+        <v>245</v>
+      </c>
+      <c r="B7" s="56" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="55" t="s">
+        <v>246</v>
+      </c>
+      <c r="D7" s="55" t="s">
+        <v>247</v>
+      </c>
+      <c r="E7" s="55" t="s">
+        <v>248</v>
+      </c>
+      <c r="F7" s="55" t="s">
+        <v>249</v>
+      </c>
     </row>
     <row r="8" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
+      <c r="A8" s="6"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
+      <c r="F8" s="6"/>
     </row>
     <row r="9" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
+      <c r="A9" s="6"/>
+      <c r="B9" s="6"/>
+      <c r="C9" s="6"/>
+      <c r="D9" s="6"/>
+      <c r="E9" s="6"/>
+      <c r="F9" s="6"/>
     </row>
     <row r="10" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
+      <c r="A10" s="6"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
+      <c r="F10" s="6"/>
     </row>
     <row r="11" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="6"/>
+      <c r="C11" s="6"/>
+      <c r="D11" s="6"/>
+      <c r="E11" s="6"/>
+      <c r="F11" s="6"/>
     </row>
     <row r="12" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
+      <c r="A12" s="6"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6"/>
     </row>
     <row r="13" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
+      <c r="A13" s="6"/>
+      <c r="B13" s="6"/>
+      <c r="C13" s="6"/>
+      <c r="D13" s="6"/>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
     </row>
     <row r="14" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
+      <c r="A14" s="6"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
     </row>
     <row r="15" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="7"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
+      <c r="A15" s="6"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
     </row>
     <row r="16" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
+      <c r="A16" s="6"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
     </row>
     <row r="17" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
+      <c r="A17" s="6"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
     </row>
     <row r="18" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
+      <c r="A18" s="6"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
     </row>
     <row r="19" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="7"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
+      <c r="A19" s="6"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
     </row>
     <row r="20" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
+      <c r="A20" s="6"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
     </row>
     <row r="21" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="7"/>
-      <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
+      <c r="A21" s="6"/>
+      <c r="B21" s="6"/>
+      <c r="C21" s="6"/>
+      <c r="D21" s="6"/>
+      <c r="E21" s="6"/>
+      <c r="F21" s="6"/>
     </row>
     <row r="22" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="7"/>
-      <c r="B22" s="7"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
+      <c r="A22" s="6"/>
+      <c r="B22" s="6"/>
+      <c r="C22" s="6"/>
+      <c r="D22" s="6"/>
+      <c r="E22" s="6"/>
+      <c r="F22" s="6"/>
     </row>
     <row r="23" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="7"/>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="7"/>
-      <c r="F23" s="7"/>
+      <c r="A23" s="6"/>
+      <c r="B23" s="6"/>
+      <c r="C23" s="6"/>
+      <c r="D23" s="6"/>
+      <c r="E23" s="6"/>
+      <c r="F23" s="6"/>
     </row>
     <row r="24" spans="1:6" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="7"/>
-      <c r="B24" s="7"/>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
-      <c r="F24" s="7"/>
+      <c r="A24" s="6"/>
+      <c r="B24" s="6"/>
+      <c r="C24" s="6"/>
+      <c r="D24" s="6"/>
+      <c r="E24" s="6"/>
+      <c r="F24" s="6"/>
     </row>
     <row r="30" spans="1:6" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
@@ -2476,68 +3080,68 @@
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" s="10" t="s">
+      <c r="A31" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="B31" s="8" t="s">
         <v>50</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C31" s="8" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="A32" s="7" t="s">
+      <c r="A32" s="6" t="s">
         <v>47</v>
       </c>
-      <c r="B32" s="7" t="s">
+      <c r="B32" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="C32" s="7" t="s">
+      <c r="C32" s="6" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="33" spans="1:3" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="A33" s="7" t="s">
+      <c r="A33" s="6" t="s">
         <v>54</v>
       </c>
-      <c r="B33" s="7" t="s">
+      <c r="B33" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="C33" s="7" t="s">
+      <c r="C33" s="6" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="34" spans="1:3" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="A34" s="7" t="s">
+      <c r="A34" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B34" s="7" t="s">
+      <c r="B34" s="6" t="s">
         <v>58</v>
       </c>
-      <c r="C34" s="7" t="s">
+      <c r="C34" s="6" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="35" spans="1:3" ht="27.6" x14ac:dyDescent="0.25">
-      <c r="A35" s="7" t="s">
+      <c r="A35" s="6" t="s">
         <v>60</v>
       </c>
-      <c r="B35" s="7" t="s">
+      <c r="B35" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="C35" s="7" t="s">
+      <c r="C35" s="6" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="36" spans="1:3" ht="41.4" x14ac:dyDescent="0.25">
-      <c r="A36" s="7" t="s">
+      <c r="A36" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B36" s="7" t="s">
+      <c r="B36" s="6" t="s">
         <v>64</v>
       </c>
-      <c r="C36" s="7" t="s">
+      <c r="C36" s="6" t="s">
         <v>65</v>
       </c>
     </row>
@@ -2552,310 +3156,375 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:D33"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8" customWidth="1"/>
-    <col min="2" max="2" width="60" customWidth="1"/>
-    <col min="3" max="3" width="10" customWidth="1"/>
-    <col min="4" max="4" width="30" customWidth="1"/>
+    <col min="1" max="1" width="8" style="30" customWidth="1"/>
+    <col min="2" max="2" width="60" style="30" customWidth="1"/>
+    <col min="3" max="3" width="10" style="30" customWidth="1"/>
+    <col min="4" max="4" width="30" style="30" customWidth="1"/>
+    <col min="5" max="16384" width="8.796875" style="30"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A1" s="20" t="s">
+      <c r="A1" s="57" t="s">
         <v>66</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="23" t="s">
+      <c r="A2" s="58" t="s">
         <v>67</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-    </row>
-    <row r="4" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A4" s="1" t="s">
+      <c r="B2" s="17"/>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+    </row>
+    <row r="4" spans="1:4" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="31" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="6" t="s">
+      <c r="A5" s="32" t="s">
         <v>69</v>
       </c>
-      <c r="B5" s="11" t="s">
+      <c r="B5" s="35" t="s">
         <v>70</v>
       </c>
-      <c r="C5" s="6" t="s">
+      <c r="C5" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D5" s="35" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="36" t="s">
         <v>73</v>
       </c>
-      <c r="B6" s="13" t="s">
+      <c r="B6" s="37" t="s">
         <v>74</v>
       </c>
-      <c r="C6" s="34" t="s">
+      <c r="C6" s="36" t="s">
         <v>75</v>
       </c>
-      <c r="D6" s="13"/>
+      <c r="D6" s="37"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="12" t="s">
+      <c r="A7" s="36" t="s">
         <v>76</v>
       </c>
-      <c r="B7" s="13" t="s">
+      <c r="B7" s="37" t="s">
         <v>77</v>
       </c>
-      <c r="C7" s="34" t="s">
+      <c r="C7" s="36" t="s">
         <v>75</v>
       </c>
-      <c r="D7" s="13"/>
+      <c r="D7" s="37"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="36" t="s">
         <v>78</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="B8" s="37" t="s">
         <v>79</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="36" t="s">
         <v>75</v>
       </c>
-      <c r="D8" s="13"/>
+      <c r="D8" s="37"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="36" t="s">
         <v>80</v>
       </c>
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="37" t="s">
         <v>81</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="36" t="s">
         <v>75</v>
       </c>
-      <c r="D9" s="13"/>
+      <c r="D9" s="37"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="36" t="s">
         <v>82</v>
       </c>
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="37" t="s">
         <v>83</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="36" t="s">
         <v>75</v>
       </c>
-      <c r="D10" s="13"/>
-    </row>
-    <row r="12" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A12" s="1" t="s">
+      <c r="D10" s="37"/>
+    </row>
+    <row r="12" spans="1:4" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="31" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A13" s="6" t="s">
+      <c r="A13" s="32" t="s">
         <v>69</v>
       </c>
-      <c r="B13" s="11" t="s">
+      <c r="B13" s="35" t="s">
         <v>70</v>
       </c>
-      <c r="C13" s="6" t="s">
+      <c r="C13" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="D13" s="11" t="s">
+      <c r="D13" s="35" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A14" s="12" t="s">
+    <row r="14" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A14" s="36" t="s">
         <v>73</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="37" t="s">
         <v>86</v>
       </c>
-      <c r="C14" s="12" t="s">
+      <c r="C14" s="36" t="s">
         <v>75</v>
       </c>
-      <c r="D14" s="13"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A15" s="12" t="s">
+      <c r="D14" s="37" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A15" s="36" t="s">
         <v>76</v>
       </c>
-      <c r="B15" s="13" t="s">
+      <c r="B15" s="37" t="s">
         <v>87</v>
       </c>
-      <c r="C15" s="12" t="s">
+      <c r="C15" s="36" t="s">
         <v>75</v>
       </c>
-      <c r="D15" s="13"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A16" s="12" t="s">
+      <c r="D15" s="37" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A16" s="36" t="s">
         <v>78</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="B16" s="37" t="s">
         <v>88</v>
       </c>
-      <c r="C16" s="12" t="s">
+      <c r="C16" s="36" t="s">
         <v>75</v>
       </c>
-      <c r="D16" s="13"/>
+      <c r="D16" s="37" t="s">
+        <v>252</v>
+      </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A17" s="12" t="s">
+      <c r="A17" s="36" t="s">
         <v>80</v>
       </c>
-      <c r="B17" s="13" t="s">
+      <c r="B17" s="37" t="s">
         <v>89</v>
       </c>
-      <c r="C17" s="12" t="s">
+      <c r="C17" s="36" t="s">
         <v>75</v>
       </c>
-      <c r="D17" s="13"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A18" s="12" t="s">
+      <c r="D17" s="37"/>
+    </row>
+    <row r="18" spans="1:4" ht="26.4" x14ac:dyDescent="0.25">
+      <c r="A18" s="36" t="s">
         <v>82</v>
       </c>
-      <c r="B18" s="13" t="s">
+      <c r="B18" s="37" t="s">
         <v>90</v>
       </c>
-      <c r="C18" s="12" t="s">
+      <c r="C18" s="36" t="s">
         <v>75</v>
       </c>
-      <c r="D18" s="13"/>
-    </row>
-    <row r="20" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="14" t="s">
+      <c r="D18" s="37" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="38" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="15" t="s">
+      <c r="A21" s="39" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="15" t="s">
+      <c r="A22" s="39" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="25" spans="1:4" ht="17.399999999999999" x14ac:dyDescent="0.3">
-      <c r="A25" s="1" t="s">
+    <row r="25" spans="1:4" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A25" s="31" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="16" t="s">
+      <c r="A26" s="40" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="27" spans="1:4" ht="55.2" x14ac:dyDescent="0.25">
-      <c r="A27" s="17" t="s">
+    <row r="27" spans="1:4" ht="55.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="41" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="10" t="s">
+      <c r="B27" s="34" t="s">
         <v>96</v>
       </c>
-      <c r="C27" s="10" t="s">
+      <c r="C27" s="34" t="s">
         <v>97</v>
       </c>
-      <c r="D27" s="10" t="s">
+      <c r="D27" s="34" t="s">
         <v>98</v>
       </c>
     </row>
-    <row r="28" spans="1:4" ht="92.4" x14ac:dyDescent="0.25">
-      <c r="A28" s="31" t="s">
+    <row r="28" spans="1:4" ht="92.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="44" t="s">
         <v>34</v>
       </c>
-      <c r="B28" s="32" t="s">
+      <c r="B28" s="45" t="s">
         <v>168</v>
       </c>
-      <c r="C28" s="32" t="s">
+      <c r="C28" s="45" t="s">
         <v>169</v>
       </c>
-      <c r="D28" s="33" t="s">
+      <c r="D28" s="46" t="s">
         <v>170</v>
       </c>
     </row>
-    <row r="29" spans="1:4" ht="105.6" x14ac:dyDescent="0.25">
-      <c r="A29" s="31" t="s">
+    <row r="29" spans="1:4" ht="105.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="44" t="s">
         <v>35</v>
       </c>
-      <c r="B29" s="32" t="s">
+      <c r="B29" s="45" t="s">
         <v>171</v>
       </c>
-      <c r="C29" s="32" t="s">
+      <c r="C29" s="45" t="s">
         <v>172</v>
       </c>
-      <c r="D29" s="33" t="s">
+      <c r="D29" s="46" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="30" spans="1:4" ht="118.8" x14ac:dyDescent="0.25">
-      <c r="A30" s="31" t="s">
+    <row r="30" spans="1:4" ht="118.8" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="44" t="s">
         <v>37</v>
       </c>
-      <c r="B30" s="32" t="s">
+      <c r="B30" s="45" t="s">
         <v>174</v>
       </c>
-      <c r="C30" s="32" t="s">
+      <c r="C30" s="45" t="s">
         <v>175</v>
       </c>
-      <c r="D30" s="33" t="s">
+      <c r="D30" s="46" t="s">
         <v>176</v>
       </c>
     </row>
-    <row r="31" spans="1:4" ht="92.4" x14ac:dyDescent="0.25">
-      <c r="A31" s="31" t="s">
+    <row r="31" spans="1:4" ht="92.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="44" t="s">
         <v>177</v>
       </c>
-      <c r="B31" s="32" t="s">
+      <c r="B31" s="45" t="s">
         <v>178</v>
       </c>
-      <c r="C31" s="32" t="s">
+      <c r="C31" s="45" t="s">
         <v>179</v>
       </c>
-      <c r="D31" s="33" t="s">
+      <c r="D31" s="46" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="32" spans="1:4" ht="79.2" x14ac:dyDescent="0.25">
-      <c r="A32" s="31" t="s">
+    <row r="32" spans="1:4" ht="79.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="44" t="s">
         <v>158</v>
       </c>
-      <c r="B32" s="32" t="s">
+      <c r="B32" s="45" t="s">
         <v>181</v>
       </c>
-      <c r="C32" s="32" t="s">
+      <c r="C32" s="45" t="s">
         <v>182</v>
       </c>
-      <c r="D32" s="33" t="s">
+      <c r="D32" s="46" t="s">
         <v>183</v>
       </c>
     </row>
-    <row r="33" spans="1:4" ht="92.4" x14ac:dyDescent="0.25">
-      <c r="A33" s="31" t="s">
+    <row r="33" spans="1:4" ht="92.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="44" t="s">
         <v>163</v>
       </c>
-      <c r="B33" s="32" t="s">
+      <c r="B33" s="45" t="s">
         <v>184</v>
       </c>
-      <c r="C33" s="32" t="s">
+      <c r="C33" s="45" t="s">
         <v>185</v>
       </c>
-      <c r="D33" s="33" t="s">
+      <c r="D33" s="46" t="s">
         <v>186</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" ht="118.8" x14ac:dyDescent="0.25">
+      <c r="A34" s="48" t="s">
+        <v>254</v>
+      </c>
+      <c r="B34" s="47" t="s">
+        <v>255</v>
+      </c>
+      <c r="C34" s="51" t="s">
+        <v>256</v>
+      </c>
+      <c r="D34" s="52" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" ht="105.6" x14ac:dyDescent="0.25">
+      <c r="A35" s="49" t="s">
+        <v>258</v>
+      </c>
+      <c r="B35" s="50" t="s">
+        <v>259</v>
+      </c>
+      <c r="C35" s="53" t="s">
+        <v>260</v>
+      </c>
+      <c r="D35" s="54" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" ht="132" x14ac:dyDescent="0.25">
+      <c r="A36" s="48" t="s">
+        <v>262</v>
+      </c>
+      <c r="B36" s="47" t="s">
+        <v>263</v>
+      </c>
+      <c r="C36" s="51" t="s">
+        <v>264</v>
+      </c>
+      <c r="D36" s="52" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" ht="145.19999999999999" x14ac:dyDescent="0.25">
+      <c r="A37" s="49" t="s">
+        <v>245</v>
+      </c>
+      <c r="B37" s="50" t="s">
+        <v>266</v>
+      </c>
+      <c r="C37" s="53" t="s">
+        <v>267</v>
+      </c>
+      <c r="D37" s="54" t="s">
+        <v>268</v>
       </c>
     </row>
   </sheetData>

</xml_diff>